<commit_message>
sku mapping module completed
</commit_message>
<xml_diff>
--- a/public/uploads/excel-formats/sku-mapping.xlsx
+++ b/public/uploads/excel-formats/sku-mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\headquater\public\uploads\excel-formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECHNOFRA-SAHIL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,70 +14,51 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>Product SKU</t>
-  </si>
-  <si>
-    <t>Customer SKU</t>
-  </si>
-  <si>
-    <t>Vendor SKU</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>Portal Code</t>
+  </si>
+  <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>Basic Rate</t>
+  </si>
+  <si>
+    <t>Net Landing Rate</t>
+  </si>
+  <si>
+    <t>MRP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF222222"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -85,35 +66,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -391,32 +352,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
-    <col min="4" max="4" width="66.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>